<commit_message>
10th commit in testing-updated deliverable files.
</commit_message>
<xml_diff>
--- a/IAC IP25 - Machine Learning - Lessons Learnt Log - Pranay Sunil Jagtap.xlsx
+++ b/IAC IP25 - Machine Learning - Lessons Learnt Log - Pranay Sunil Jagtap.xlsx
@@ -790,9 +790,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>1459800</xdr:colOff>
+      <xdr:colOff>1459440</xdr:colOff>
       <xdr:row>6</xdr:row>
-      <xdr:rowOff>18000</xdr:rowOff>
+      <xdr:rowOff>17640</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -807,7 +807,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="250560"/>
-          <a:ext cx="2673360" cy="940320"/>
+          <a:ext cx="2673000" cy="939960"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>

</xml_diff>